<commit_message>
Extensor test done and sns simulink gui
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_20mm.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_20mm.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80079B6-147F-4019-8A3C-DB46FCEA998C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D541CE-E7A5-4DC6-B614-B6F65C853A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest40mm_1" sheetId="1" r:id="rId1"/>
     <sheet name="ExtTest40mm_2" sheetId="2" r:id="rId2"/>
     <sheet name="ExtTest20mm_1" sheetId="10" r:id="rId3"/>
-    <sheet name="ExtTest20mm_2" sheetId="3" r:id="rId4"/>
+    <sheet name="ExtTest20mm_2" sheetId="11" r:id="rId4"/>
     <sheet name="FlxTest20mm_42cm" sheetId="4" r:id="rId5"/>
     <sheet name="FlxTest20mm_39cm" sheetId="5" r:id="rId6"/>
     <sheet name="FlxTest20mm_39cm (2)" sheetId="6" r:id="rId7"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="60">
   <si>
     <t>Flexor Test 20mm</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>Torque at t1</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -1237,7 +1240,14 @@
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
-  <c:style val="2"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1288,13 +1298,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>10</c:v>
+                  <c:v>-26.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11</c:v>
+                  <c:v>-30</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>-61</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-43</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-119</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1306,22 +1325,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>1.0381838898090796</c:v>
+                  <c:v>43.460736823868544</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.9717875622415679</c:v>
+                  <c:v>44.185666386660522</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.758112821237887</c:v>
+                  <c:v>41.376763734939175</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>43.865492956682836</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>29.094426649018608</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>24.781100465532006</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1377,7 +1396,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FE37-4FC1-8A2D-AAA215DD1B14}"/>
+              <c16:uniqueId val="{00000000-024E-4B50-9FEF-6C2014DD174B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4569,11 +4588,13 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A51F9805-328B-4D57-BA65-7B91B7B89C3E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -7440,8 +7461,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:X21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA2ABF78-C1E8-448F-AF95-D36F16313176}">
+  <dimension ref="A1:X28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" customWidth="1"/>
@@ -7577,17 +7598,23 @@
         <v>8</v>
       </c>
       <c r="C6" s="36">
-        <v>3.7</v>
+        <v>180.2</v>
       </c>
       <c r="D6" s="36">
-        <v>25.2</v>
+        <v>181.5</v>
       </c>
       <c r="E6" s="36">
-        <v>76</v>
-      </c>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
+        <v>168</v>
+      </c>
+      <c r="F6" s="36">
+        <v>181</v>
+      </c>
+      <c r="G6" s="36">
+        <v>116</v>
+      </c>
+      <c r="H6" s="36">
+        <v>100</v>
+      </c>
       <c r="I6" s="36"/>
       <c r="J6" s="36"/>
       <c r="K6" s="36"/>
@@ -7610,17 +7637,23 @@
         <v>9</v>
       </c>
       <c r="C7" s="37">
-        <v>10</v>
+        <v>-26.2</v>
       </c>
       <c r="D7" s="37">
-        <v>11</v>
+        <v>-30</v>
       </c>
       <c r="E7" s="37">
-        <v>10</v>
-      </c>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
+        <v>-61</v>
+      </c>
+      <c r="F7" s="37">
+        <v>-43</v>
+      </c>
+      <c r="G7" s="37">
+        <v>-119</v>
+      </c>
+      <c r="H7" s="37">
+        <v>5</v>
+      </c>
       <c r="I7" s="37"/>
       <c r="J7" s="37"/>
       <c r="K7" s="37"/>
@@ -7643,17 +7676,23 @@
         <v>10</v>
       </c>
       <c r="C8" s="38">
-        <v>388.5</v>
+        <v>437</v>
       </c>
       <c r="D8" s="38">
-        <v>388</v>
+        <v>420</v>
       </c>
       <c r="E8" s="38">
-        <v>592</v>
-      </c>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="38"/>
+        <v>425</v>
+      </c>
+      <c r="F8" s="38">
+        <v>435</v>
+      </c>
+      <c r="G8" s="38">
+        <v>256</v>
+      </c>
+      <c r="H8" s="38">
+        <v>480</v>
+      </c>
       <c r="I8" s="38"/>
       <c r="J8" s="38"/>
       <c r="K8" s="38"/>
@@ -7706,17 +7745,23 @@
         <v>13</v>
       </c>
       <c r="C10" s="37">
-        <v>72.5</v>
+        <v>28</v>
       </c>
       <c r="D10" s="37">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="E10" s="37">
-        <v>68</v>
-      </c>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
+        <v>23</v>
+      </c>
+      <c r="F10" s="37">
+        <v>27</v>
+      </c>
+      <c r="G10" s="37">
+        <v>10.5</v>
+      </c>
+      <c r="H10" s="37">
+        <v>21</v>
+      </c>
       <c r="I10" s="37"/>
       <c r="J10" s="37"/>
       <c r="K10" s="37"/>
@@ -7796,70 +7841,70 @@
         <v>17</v>
       </c>
       <c r="C13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="D13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="E13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="F13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="G13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="H13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="I13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="J13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="K13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="L13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="M13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="N13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="O13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="P13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="Q13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="R13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="S13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="T13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="U13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="V13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="W13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
       <c r="X13" s="37">
-        <v>292.89999999999998</v>
+        <v>250.9</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.3">
@@ -7921,28 +7966,28 @@
         <v>58</v>
       </c>
       <c r="C16" s="36">
-        <f>C6*SIN(RADIANS(C10+0.83))*C13/1000</f>
-        <v>1.0381838898090796</v>
+        <f>C6*COS(RADIANS(C10-12))*C13/1000</f>
+        <v>43.460736823868544</v>
       </c>
       <c r="D16" s="36">
-        <f t="shared" ref="D16:X16" si="0">D6*SIN(RADIANS(D10+0.83))*D13/1000</f>
-        <v>6.9717875622415679</v>
+        <f t="shared" ref="D16:X16" si="0">D6*COS(RADIANS(D10-12))*D13/1000</f>
+        <v>44.185666386660522</v>
       </c>
       <c r="E16" s="36">
         <f t="shared" si="0"/>
-        <v>20.758112821237887</v>
+        <v>41.376763734939175</v>
       </c>
       <c r="F16" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>43.865492956682836</v>
       </c>
       <c r="G16" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>29.094426649018608</v>
       </c>
       <c r="H16" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>24.781100465532006</v>
       </c>
       <c r="I16" s="36">
         <f t="shared" si="0"/>
@@ -8016,9 +8061,15 @@
       <c r="C17" s="37"/>
       <c r="D17" s="37"/>
       <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
+      <c r="F17" s="37">
+        <v>50.58</v>
+      </c>
+      <c r="G17" s="37">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="H17" s="37">
+        <v>28.8</v>
+      </c>
       <c r="I17" s="37"/>
       <c r="J17" s="37"/>
       <c r="K17" s="37"/>
@@ -8042,6 +8093,11 @@
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="F28" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sns modeling and torque paper
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_20mm.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_20mm.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D541CE-E7A5-4DC6-B614-B6F65C853A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8126D7CE-AF2D-48BF-9724-9E75033E0C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32505" yWindow="2760" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest40mm_1" sheetId="1" r:id="rId1"/>
@@ -1325,22 +1325,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>43.460736823868544</c:v>
+                  <c:v>46.079253454685158</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>44.185666386660522</c:v>
+                  <c:v>46.778257041650242</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>41.376763734939175</c:v>
+                  <c:v>43.708827289351646</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>43.865492956682836</c:v>
+                  <c:v>46.473685245945447</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>29.094426649018608</c:v>
+                  <c:v>30.464076188718234</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>24.781100465532006</c:v>
+                  <c:v>26.140251495852954</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5155,24 +5155,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -5180,7 +5180,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -5201,7 +5201,7 @@
         <v>0.17953321364452424</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>24</v>
       </c>
@@ -5215,7 +5215,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -5265,7 +5265,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
@@ -5312,7 +5312,7 @@
         <v>19.314</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -5359,7 +5359,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>32.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
@@ -5457,7 +5457,7 @@
         <v>33.5</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>14</v>
@@ -5505,7 +5505,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>27</v>
@@ -5567,7 +5567,7 @@
         <v>0.22800718132854578</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
@@ -5575,7 +5575,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>17</v>
@@ -5626,7 +5626,7 @@
         <v>366.05</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>18</v>
@@ -5674,13 +5674,13 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -5745,22 +5745,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
       <c r="J17" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O18" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
         <v>22</v>
       </c>
@@ -5768,7 +5768,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C21">
         <v>6.1297215268519301</v>
       </c>
@@ -5776,7 +5776,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C22">
         <v>2.7479725044346299</v>
       </c>
@@ -5790,7 +5790,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C23">
         <v>1.5877091527759399</v>
       </c>
@@ -5804,12 +5804,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C24">
         <v>0.39396830053809201</v>
       </c>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C25">
         <v>0.87997523971335201</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C26">
         <v>1.3017605698980601</v>
       </c>
@@ -5831,7 +5831,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C27">
         <v>0.32710826122173697</v>
       </c>
@@ -5845,37 +5845,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C28">
         <v>5.7663175704745298</v>
       </c>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C29">
         <v>0.99793195771798704</v>
       </c>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C30">
         <v>1.17473937755851</v>
       </c>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C31">
         <v>5.6669972560913404</v>
       </c>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C32">
         <v>3.0532323371378101</v>
       </c>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33">
         <v>9.8822570388584001</v>
       </c>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34">
         <v>5.8339811315985299</v>
       </c>
@@ -5890,29 +5890,29 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:X21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -5928,7 +5928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B5" s="24" t="s">
         <v>7</v>
       </c>
@@ -5999,7 +5999,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B6" s="13" t="s">
         <v>8</v>
       </c>
@@ -6026,7 +6026,7 @@
       <c r="W6" s="36"/>
       <c r="X6" s="36"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
         <v>9</v>
       </c>
@@ -6053,7 +6053,7 @@
       <c r="W7" s="37"/>
       <c r="X7" s="37"/>
     </row>
-    <row r="8" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>10</v>
       </c>
@@ -6080,7 +6080,7 @@
       <c r="W8" s="38"/>
       <c r="X8" s="38"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>11</v>
       </c>
@@ -6110,7 +6110,7 @@
       <c r="W9" s="36"/>
       <c r="X9" s="36"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
@@ -6137,7 +6137,7 @@
       <c r="W10" s="37"/>
       <c r="X10" s="37"/>
     </row>
-    <row r="11" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
         <v>14</v>
       </c>
@@ -6164,7 +6164,7 @@
       <c r="W11" s="38"/>
       <c r="X11" s="38"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>15</v>
       </c>
@@ -6194,7 +6194,7 @@
       <c r="W12" s="36"/>
       <c r="X12" s="36"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>17</v>
       </c>
@@ -6221,7 +6221,7 @@
       <c r="W13" s="37"/>
       <c r="X13" s="37"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>18</v>
       </c>
@@ -6248,7 +6248,7 @@
       <c r="W14" s="37"/>
       <c r="X14" s="37"/>
     </row>
-    <row r="15" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="28" t="s">
         <v>19</v>
       </c>
@@ -6275,7 +6275,7 @@
       <c r="W15" s="38"/>
       <c r="X15" s="38"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B16" s="13" t="s">
         <v>20</v>
       </c>
@@ -6368,7 +6368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -6395,7 +6395,7 @@
       <c r="W17" s="36"/>
       <c r="X17" s="36"/>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -6412,24 +6412,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Q27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -6437,7 +6437,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v>462.31</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>24</v>
       </c>
@@ -6454,7 +6454,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
@@ -6515,7 +6515,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -6526,7 +6526,7 @@
         <v>-16</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>35</v>
       </c>
@@ -6537,7 +6537,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -6548,7 +6548,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>13</v>
@@ -6599,7 +6599,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>14</v>
@@ -6608,7 +6608,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>36</v>
@@ -6618,7 +6618,7 @@
         <v>0.28366247755834828</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>15</v>
       </c>
@@ -6626,7 +6626,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>17</v>
@@ -6677,7 +6677,7 @@
         <v>240.61</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
       <c r="B15" s="8" t="s">
         <v>18</v>
@@ -6686,13 +6686,13 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
         <v>20</v>
       </c>
@@ -6757,7 +6757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>37</v>
       </c>
@@ -6768,12 +6768,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>31</v>
       </c>
@@ -6784,7 +6784,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>32</v>
       </c>
@@ -6802,7 +6802,7 @@
         <v>18.260899999999999</v>
       </c>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C23">
         <v>2.018E-2</v>
       </c>
@@ -6813,12 +6813,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>32</v>
       </c>
@@ -6832,7 +6832,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C27">
         <v>3.619E-2</v>
       </c>
@@ -6852,19 +6852,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{411EFBF4-5987-49CA-839E-BE22E507CBB9}">
   <dimension ref="A1:X21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>41</v>
       </c>
@@ -6887,12 +6887,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -6903,7 +6903,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="24" t="s">
         <v>7</v>
       </c>
@@ -6982,7 +6982,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B6" s="13" t="s">
         <v>8</v>
       </c>
@@ -7015,7 +7015,7 @@
       <c r="W6" s="36"/>
       <c r="X6" s="36"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
         <v>9</v>
       </c>
@@ -7048,7 +7048,7 @@
       <c r="W7" s="37"/>
       <c r="X7" s="37"/>
     </row>
-    <row r="8" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>10</v>
       </c>
@@ -7081,7 +7081,7 @@
       <c r="W8" s="38"/>
       <c r="X8" s="38"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>11</v>
       </c>
@@ -7111,7 +7111,7 @@
       <c r="W9" s="36"/>
       <c r="X9" s="36"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
@@ -7144,7 +7144,7 @@
       <c r="W10" s="37"/>
       <c r="X10" s="37"/>
     </row>
-    <row r="11" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
         <v>14</v>
       </c>
@@ -7171,7 +7171,7 @@
       <c r="W11" s="38"/>
       <c r="X11" s="38"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>15</v>
       </c>
@@ -7201,7 +7201,7 @@
       <c r="W12" s="36"/>
       <c r="X12" s="36"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>17</v>
       </c>
@@ -7272,7 +7272,7 @@
         <v>292.89999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>18</v>
       </c>
@@ -7299,7 +7299,7 @@
       <c r="W14" s="37"/>
       <c r="X14" s="37"/>
     </row>
-    <row r="15" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="28" t="s">
         <v>19</v>
       </c>
@@ -7326,7 +7326,7 @@
       <c r="W15" s="38"/>
       <c r="X15" s="38"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>58</v>
       </c>
@@ -7419,7 +7419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -7446,7 +7446,7 @@
       <c r="W17" s="37"/>
       <c r="X17" s="37"/>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -7463,19 +7463,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA2ABF78-C1E8-448F-AF95-D36F16313176}">
   <dimension ref="A1:X28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>41</v>
       </c>
@@ -7498,12 +7498,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -7514,7 +7514,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -7522,7 +7522,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="24" t="s">
         <v>7</v>
       </c>
@@ -7593,7 +7593,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B6" s="13" t="s">
         <v>8</v>
       </c>
@@ -7632,7 +7632,7 @@
       <c r="W6" s="36"/>
       <c r="X6" s="36"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
         <v>9</v>
       </c>
@@ -7671,7 +7671,7 @@
       <c r="W7" s="37"/>
       <c r="X7" s="37"/>
     </row>
-    <row r="8" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>10</v>
       </c>
@@ -7710,7 +7710,7 @@
       <c r="W8" s="38"/>
       <c r="X8" s="38"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>11</v>
       </c>
@@ -7740,7 +7740,7 @@
       <c r="W9" s="36"/>
       <c r="X9" s="36"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
@@ -7779,7 +7779,7 @@
       <c r="W10" s="37"/>
       <c r="X10" s="37"/>
     </row>
-    <row r="11" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
         <v>14</v>
       </c>
@@ -7806,7 +7806,7 @@
       <c r="W11" s="38"/>
       <c r="X11" s="38"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>15</v>
       </c>
@@ -7836,78 +7836,78 @@
       <c r="W12" s="36"/>
       <c r="X12" s="36"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="D13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="E13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="F13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="G13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="H13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="I13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="J13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="K13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="L13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="M13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="N13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="O13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="P13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="Q13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="R13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="S13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="T13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="U13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="V13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="W13" s="37">
-        <v>250.9</v>
+        <v>263.2</v>
       </c>
       <c r="X13" s="37">
-        <v>250.9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+        <v>263.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>18</v>
       </c>
@@ -7934,7 +7934,7 @@
       <c r="W14" s="37"/>
       <c r="X14" s="37"/>
     </row>
-    <row r="15" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="28" t="s">
         <v>19</v>
       </c>
@@ -7961,33 +7961,33 @@
       <c r="W15" s="38"/>
       <c r="X15" s="38"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>58</v>
       </c>
       <c r="C16" s="36">
-        <f>C6*COS(RADIANS(C10-12))*C13/1000</f>
-        <v>43.460736823868544</v>
+        <f>C6*COS(RADIANS(C10-14.3))*C13/1000</f>
+        <v>46.079253454685158</v>
       </c>
       <c r="D16" s="36">
-        <f t="shared" ref="D16:X16" si="0">D6*COS(RADIANS(D10-12))*D13/1000</f>
-        <v>44.185666386660522</v>
+        <f t="shared" ref="D16:X16" si="0">D6*COS(RADIANS(D10-14.3))*D13/1000</f>
+        <v>46.778257041650242</v>
       </c>
       <c r="E16" s="36">
         <f t="shared" si="0"/>
-        <v>41.376763734939175</v>
+        <v>43.708827289351646</v>
       </c>
       <c r="F16" s="36">
         <f t="shared" si="0"/>
-        <v>43.865492956682836</v>
+        <v>46.473685245945447</v>
       </c>
       <c r="G16" s="36">
         <f t="shared" si="0"/>
-        <v>29.094426649018608</v>
+        <v>30.464076188718234</v>
       </c>
       <c r="H16" s="36">
         <f t="shared" si="0"/>
-        <v>24.781100465532006</v>
+        <v>26.140251495852954</v>
       </c>
       <c r="I16" s="36">
         <f t="shared" si="0"/>
@@ -8054,7 +8054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -8087,7 +8087,7 @@
       <c r="W17" s="37"/>
       <c r="X17" s="37"/>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -8095,7 +8095,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:24" x14ac:dyDescent="0.25">
       <c r="F28" t="s">
         <v>59</v>
       </c>
@@ -8109,24 +8109,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -8134,7 +8134,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -8157,7 +8157,7 @@
         <v>0.12647754137115841</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -8174,7 +8174,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -8230,7 +8230,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
@@ -8286,7 +8286,7 @@
         <v>4.8666</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -8342,7 +8342,7 @@
         <v>-120</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>10</v>
       </c>
@@ -8398,7 +8398,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -8457,7 +8457,7 @@
         <v>48.1</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>13</v>
@@ -8514,7 +8514,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>14</v>
@@ -8573,7 +8573,7 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
@@ -8596,7 +8596,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>17</v>
@@ -8653,7 +8653,7 @@
         <v>366.43</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>18</v>
@@ -8710,13 +8710,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -8789,7 +8789,7 @@
         <v>-1.0937153129886135</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -8845,22 +8845,22 @@
         <v>-0.77272430551831095</v>
       </c>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="J18" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
       <c r="M19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
       <c r="R20" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -8878,24 +8878,24 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -8910,7 +8910,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -8940,7 +8940,7 @@
         <v>0.12647754137115841</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -8960,7 +8960,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -9016,7 +9016,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
@@ -9042,7 +9042,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -9068,7 +9068,7 @@
         <v>-64</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>10</v>
       </c>
@@ -9094,7 +9094,7 @@
         <v>606.5</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -9102,7 +9102,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>13</v>
@@ -9129,7 +9129,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>14</v>
@@ -9157,7 +9157,7 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
@@ -9180,7 +9180,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>17</v>
@@ -9234,7 +9234,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>18</v>
@@ -9258,13 +9258,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -9337,12 +9337,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -9360,24 +9360,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -9392,7 +9392,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -9422,7 +9422,7 @@
         <v>0.12647754137115841</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -9436,7 +9436,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -9492,7 +9492,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
@@ -9509,7 +9509,7 @@
         <v>50.45</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -9526,7 +9526,7 @@
         <v>-75</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>10</v>
       </c>
@@ -9543,7 +9543,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -9551,7 +9551,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>13</v>
@@ -9569,7 +9569,7 @@
         <v>26.5</v>
       </c>
     </row>
-    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>14</v>
@@ -9591,7 +9591,7 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
@@ -9614,7 +9614,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>17</v>
@@ -9668,7 +9668,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>18</v>
@@ -9686,13 +9686,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -9765,7 +9765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -9773,7 +9773,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -9791,24 +9791,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -9823,7 +9823,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -9844,7 +9844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -9855,7 +9855,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -9911,7 +9911,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
@@ -9940,7 +9940,7 @@
         <v>78.14</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -9969,7 +9969,7 @@
         <v>-32</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>10</v>
       </c>
@@ -9998,7 +9998,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -10006,7 +10006,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>13</v>
@@ -10036,7 +10036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>14</v>
@@ -10070,7 +10070,7 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
@@ -10093,7 +10093,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>17</v>
@@ -10147,7 +10147,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>18</v>
@@ -10177,13 +10177,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -10256,7 +10256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -10279,7 +10279,7 @@
         <v>-22.190799999999999</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
@@ -10297,24 +10297,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AD21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="9" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="13.42578125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -10329,7 +10329,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -10355,7 +10355,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:30" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
@@ -10375,7 +10375,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="27" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" s="27" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23"/>
       <c r="B5" s="24" t="s">
         <v>7</v>
@@ -10465,7 +10465,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B6" s="13" t="s">
         <v>8</v>
       </c>
@@ -10536,7 +10536,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
         <v>9</v>
       </c>
@@ -10607,7 +10607,7 @@
         <v>-32</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="32" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" s="32" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="28"/>
       <c r="B8" s="29" t="s">
         <v>10</v>
@@ -10679,7 +10679,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>11</v>
       </c>
@@ -10709,7 +10709,7 @@
       <c r="W9" s="21"/>
       <c r="X9" s="21"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="3" t="s">
         <v>13</v>
@@ -10781,7 +10781,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="34" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" s="34" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="33"/>
       <c r="B11" s="28" t="s">
         <v>14</v>
@@ -10853,7 +10853,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>15</v>
       </c>
@@ -10883,7 +10883,7 @@
       <c r="W12" s="21"/>
       <c r="X12" s="21"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
       <c r="B13" s="3" t="s">
         <v>17</v>
@@ -10973,7 +10973,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
       <c r="B14" s="3" t="s">
         <v>18</v>
@@ -11045,7 +11045,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="32" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:30" s="32" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33"/>
       <c r="B15" s="28" t="s">
         <v>19</v>
@@ -11073,7 +11073,7 @@
       <c r="W15" s="30"/>
       <c r="X15" s="30"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B16" s="13" t="s">
         <v>20</v>
       </c>
@@ -11190,7 +11190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -11261,7 +11261,7 @@
         <v>-23.6068</v>
       </c>
     </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:24" x14ac:dyDescent="0.25">
       <c r="K18" t="s">
         <v>48</v>
       </c>
@@ -11269,7 +11269,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:24" x14ac:dyDescent="0.25">
       <c r="U19" t="s">
         <v>50</v>
       </c>
@@ -11277,7 +11277,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:24" x14ac:dyDescent="0.25">
       <c r="F20" t="s">
         <v>52</v>
       </c>
@@ -11285,7 +11285,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
ran more extensor test and bipulley re-optimization
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_20mm.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_20mm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8126D7CE-AF2D-48BF-9724-9E75033E0C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FF60C62-5EE5-4E66-93DF-91FD720B36C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32505" yWindow="2760" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest40mm_1" sheetId="1" r:id="rId1"/>
@@ -1315,6 +1315,15 @@
                 <c:pt idx="5">
                   <c:v>5</c:v>
                 </c:pt>
+                <c:pt idx="6">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-22</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-86.5</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1325,31 +1334,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>46.079253454685158</c:v>
+                  <c:v>44.8113882594823</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46.778257041650242</c:v>
+                  <c:v>45.585747457333838</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>43.708827289351646</c:v>
+                  <c:v>42.724833518295966</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46.473685245945447</c:v>
+                  <c:v>45.242138509683038</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30.464076188718234</c:v>
+                  <c:v>30.146746944099203</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>26.140251495852954</c:v>
+                  <c:v>25.602991386762568</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>31.494527360331841</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>43.120392476105614</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>35.729549720172791</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -7615,9 +7624,15 @@
       <c r="H6" s="36">
         <v>100</v>
       </c>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
+      <c r="I6" s="36">
+        <v>126</v>
+      </c>
+      <c r="J6" s="36">
+        <v>173.4</v>
+      </c>
+      <c r="K6" s="36">
+        <v>140</v>
+      </c>
       <c r="L6" s="36"/>
       <c r="M6" s="36"/>
       <c r="N6" s="36"/>
@@ -7654,9 +7669,15 @@
       <c r="H7" s="37">
         <v>5</v>
       </c>
-      <c r="I7" s="37"/>
-      <c r="J7" s="37"/>
-      <c r="K7" s="37"/>
+      <c r="I7" s="37">
+        <v>-1</v>
+      </c>
+      <c r="J7" s="37">
+        <v>-22</v>
+      </c>
+      <c r="K7" s="37">
+        <v>-86.5</v>
+      </c>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
       <c r="N7" s="37"/>
@@ -7693,9 +7714,15 @@
       <c r="H8" s="38">
         <v>480</v>
       </c>
-      <c r="I8" s="38"/>
-      <c r="J8" s="38"/>
-      <c r="K8" s="38"/>
+      <c r="I8" s="38">
+        <v>488</v>
+      </c>
+      <c r="J8" s="38">
+        <v>435</v>
+      </c>
+      <c r="K8" s="38">
+        <v>350</v>
+      </c>
       <c r="L8" s="38"/>
       <c r="M8" s="38"/>
       <c r="N8" s="38"/>
@@ -7762,9 +7789,15 @@
       <c r="H10" s="37">
         <v>21</v>
       </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="37"/>
+      <c r="I10" s="37">
+        <v>27</v>
+      </c>
+      <c r="J10" s="37">
+        <v>28</v>
+      </c>
+      <c r="K10" s="37">
+        <v>22</v>
+      </c>
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
       <c r="N10" s="37"/>
@@ -7841,70 +7874,70 @@
         <v>17</v>
       </c>
       <c r="C13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="D13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="E13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="F13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="G13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="H13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="I13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="J13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="K13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="L13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="M13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="N13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="O13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="P13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="Q13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="R13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="S13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="T13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="U13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="V13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="W13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="X13" s="37">
-        <v>263.2</v>
+        <v>259.89999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
@@ -7966,40 +7999,40 @@
         <v>58</v>
       </c>
       <c r="C16" s="36">
-        <f>C6*COS(RADIANS(C10-14.3))*C13/1000</f>
-        <v>46.079253454685158</v>
+        <f>C6*COS(RADIANS(C10-11.1))*C13/1000</f>
+        <v>44.8113882594823</v>
       </c>
       <c r="D16" s="36">
-        <f t="shared" ref="D16:X16" si="0">D6*COS(RADIANS(D10-14.3))*D13/1000</f>
-        <v>46.778257041650242</v>
+        <f t="shared" ref="D16:X16" si="0">D6*COS(RADIANS(D10-11.1))*D13/1000</f>
+        <v>45.585747457333838</v>
       </c>
       <c r="E16" s="36">
         <f t="shared" si="0"/>
-        <v>43.708827289351646</v>
+        <v>42.724833518295966</v>
       </c>
       <c r="F16" s="36">
         <f t="shared" si="0"/>
-        <v>46.473685245945447</v>
+        <v>45.242138509683038</v>
       </c>
       <c r="G16" s="36">
         <f t="shared" si="0"/>
-        <v>30.464076188718234</v>
+        <v>30.146746944099203</v>
       </c>
       <c r="H16" s="36">
         <f t="shared" si="0"/>
-        <v>26.140251495852954</v>
+        <v>25.602991386762568</v>
       </c>
       <c r="I16" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>31.494527360331841</v>
       </c>
       <c r="J16" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>43.120392476105614</v>
       </c>
       <c r="K16" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35.729549720172791</v>
       </c>
       <c r="L16" s="36">
         <f t="shared" si="0"/>
@@ -8070,9 +8103,15 @@
       <c r="H17" s="37">
         <v>28.8</v>
       </c>
-      <c r="I17" s="37"/>
-      <c r="J17" s="37"/>
-      <c r="K17" s="37"/>
+      <c r="I17" s="37">
+        <v>36.86</v>
+      </c>
+      <c r="J17" s="37">
+        <v>49.95</v>
+      </c>
+      <c r="K17" s="37">
+        <v>39.71</v>
+      </c>
       <c r="L17" s="37"/>
       <c r="M17" s="37"/>
       <c r="N17" s="37"/>
@@ -8102,7 +8141,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>